<commit_message>
Algo toolbox: apply independent technical review
Fixes: Western Electric rules (consecutive, same side), I-MR notation and
MR LCL, IPS companion chapter labels, CT phases derived from tags, project
loop rebuilt so every cycle passes the term-limit check (machine-checked).
Adds: SPC constants table (A2..c4, n = 2..10, recomputed at build), test
roadmap rows (spread, McNemar, goodness of fit, Poisson), ST-LOGIT, Laney
and EWMA/CUSUM chart rows, IPS wording for t, proportion and chi-square
conditions, %GRR to tolerance, attribute agreement bands, FMEA house-rule
label, Pareto reconciliation cell. Review kept as REVIEW_FABLE.md.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VHV4X8Aiu1hbp6cXC8cgcp
</commit_message>
<xml_diff>
--- a/algo-toolbox/ALGO_TOOLBOX.xlsx
+++ b/algo-toolbox/ALGO_TOOLBOX.xlsx
@@ -36,8 +36,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="12">
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="0.000"/>
+    <numFmt numFmtId="165" formatCode="0.0000"/>
+  </numFmts>
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -106,6 +109,12 @@
       <name val="Calibri"/>
       <i val="1"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="008B0000"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="22">
@@ -262,7 +271,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="65">
+  <cellXfs count="73">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" indent="1"/>
@@ -418,6 +427,24 @@
     <xf numFmtId="0" fontId="2" fillId="20" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="1" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="3" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" indent="1"/>
     </xf>
@@ -445,6 +472,10 @@
     </xf>
     <xf numFmtId="9" fontId="4" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="21" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -693,7 +724,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>16</row>
+      <row>17</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="6660000" cy="3960000"/>
@@ -1272,28 +1303,28 @@
       </c>
     </row>
     <row r="3" ht="21" customHeight="1">
-      <c r="A3" s="63" t="inlineStr">
+      <c r="A3" s="71" t="inlineStr">
         <is>
           <t>Six Sigma methodology (owner's Six Sigma books)</t>
         </is>
       </c>
-      <c r="B3" s="64" t="inlineStr">
+      <c r="B3" s="72" t="inlineStr">
         <is>
           <t>Six Sigma, Crosswalk</t>
         </is>
       </c>
-      <c r="C3" s="64" t="inlineStr">
+      <c r="C3" s="72" t="inlineStr">
         <is>
           <t>baseline</t>
         </is>
       </c>
-      <c r="D3" s="64" t="inlineStr">
+      <c r="D3" s="72" t="inlineStr">
         <is>
           <t>Book titles and paths needed; run extract/ with --lexicon six_sigma.</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="36" customHeight="1">
+    <row r="4" ht="51" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Moore, McCabe &amp; Craig, Introduction to the Practice of Statistics</t>
@@ -1311,27 +1342,27 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Chapters are likely numbers for recent editions; verify against the owner's edition. Codex stats extraction will replace this sheet.</t>
+          <t>Chapter numbers match the 6th to 9th editions (Fable review); 10th edition believed unchanged, unverified. Chapters 14 to 17 are online companion chapters. Codex stats extraction will replace this sheet.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="21" customHeight="1">
-      <c r="A5" s="63" t="inlineStr">
+      <c r="A5" s="71" t="inlineStr">
         <is>
           <t>Owner's engineering statistics text</t>
         </is>
       </c>
-      <c r="B5" s="64" t="inlineStr">
+      <c r="B5" s="72" t="inlineStr">
         <is>
           <t>Statistics</t>
         </is>
       </c>
-      <c r="C5" s="64" t="inlineStr">
+      <c r="C5" s="72" t="inlineStr">
         <is>
           <t>pending</t>
         </is>
       </c>
-      <c r="D5" s="64" t="inlineStr">
+      <c r="D5" s="72" t="inlineStr">
         <is>
           <t>Title needed.</t>
         </is>
@@ -1359,25 +1390,25 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="21" customHeight="1">
-      <c r="A7" s="63" t="inlineStr">
-        <is>
-          <t>AIAG MSA (4th ed.) and AIAG-VDA FMEA (2019)</t>
-        </is>
-      </c>
-      <c r="B7" s="64" t="inlineStr">
-        <is>
-          <t>Six Sigma</t>
-        </is>
-      </c>
-      <c r="C7" s="64" t="inlineStr">
+    <row r="7" ht="36" customHeight="1">
+      <c r="A7" s="71" t="inlineStr">
+        <is>
+          <t>AIAG MSA (4th ed.), AIAG FMEA (4th ed.), AIAG-VDA FMEA (2019), AIAG SPC</t>
+        </is>
+      </c>
+      <c r="B7" s="72" t="inlineStr">
+        <is>
+          <t>Six Sigma, Decision Algorithms</t>
+        </is>
+      </c>
+      <c r="C7" s="72" t="inlineStr">
         <is>
           <t>baseline</t>
         </is>
       </c>
-      <c r="D7" s="64" t="inlineStr">
-        <is>
-          <t>Thresholds for %GRR, ndc, and FMEA Action Priority.</t>
+      <c r="D7" s="72" t="inlineStr">
+        <is>
+          <t>Thresholds for %GRR, ndc, attribute agreement, FMEA RPN and Action Priority; chart constants. The 1.5 shift, Cpk, %GRR and kappa bands are not from IPS.</t>
         </is>
       </c>
     </row>
@@ -1682,7 +1713,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="36" customHeight="1">
+    <row r="12" ht="51" customHeight="1">
       <c r="A12" s="26" t="inlineStr">
         <is>
           <t>Gage R&amp;R (MSA, ANOVA method)</t>
@@ -1690,7 +1721,7 @@
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>%GRR = sigma_GRR / sigma_total x 100. ndc = 1.41 x sigma_part / sigma_GRR.</t>
+          <t>%GRR = sigma_GRR / sigma_total x 100. %GRR to tolerance = 6 sigma_GRR / (USL - LSL) x 100. ndc = 1.41 x sigma_part / sigma_GRR, truncated to an integer.</t>
         </is>
       </c>
       <c r="C12" s="8" t="inlineStr">
@@ -1706,12 +1737,11 @@
       </c>
       <c r="E12" s="8" t="inlineStr">
         <is>
-          <t>One-way ANOVA (IPS ch. 12)
-Two-way ANOVA (IPS ch. 13)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="36" customHeight="1">
+          <t>Two-way ANOVA (IPS ch. 13)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="66" customHeight="1">
       <c r="A13" s="26" t="inlineStr">
         <is>
           <t>Attribute agreement analysis</t>
@@ -1724,7 +1754,7 @@
       </c>
       <c r="C13" s="8" t="inlineStr">
         <is>
-          <t>kappa &gt;= 0.75 good; 0.40 to 0.75 marginal; &lt; 0.40 poor.</t>
+          <t>kappa &gt;= 0.75 good; 0.40 to 0.75 marginal; &lt; 0.40 poor. AIAG: effectiveness &gt;= 90%, miss rate &lt;= 2%, false alarm &lt;= 5%. A chi-square test shows association, not agreement.</t>
         </is>
       </c>
       <c r="D13" s="8" t="inlineStr">
@@ -1734,11 +1764,11 @@
       </c>
       <c r="E13" s="8" t="inlineStr">
         <is>
-          <t>Chi-square test for two-way tables (IPS ch. 9)</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="36" customHeight="1">
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="51" customHeight="1">
       <c r="A14" s="26" t="inlineStr">
         <is>
           <t>Normality check</t>
@@ -1751,7 +1781,7 @@
       </c>
       <c r="C14" s="8" t="inlineStr">
         <is>
-          <t>p &gt; alpha and a straight plot -&gt; treat as normal; else transform or go nonparametric.</t>
+          <t>p &gt; alpha means no evidence against normality; decide from the plot. Large n: rely on the plot. Small n: the test has little power.</t>
         </is>
       </c>
       <c r="D14" s="8" t="inlineStr">
@@ -1766,7 +1796,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="51" customHeight="1">
+    <row r="15" ht="66" customHeight="1">
       <c r="A15" s="26" t="inlineStr">
         <is>
           <t>Baseline capability</t>
@@ -1774,12 +1804,12 @@
       </c>
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t>Cp = (USL - LSL) / 6 sigma_within. Cpk = min(USL - mean, mean - LSL) / 3 sigma_within. Pp, Ppk use overall sigma.</t>
+          <t>Cp = (USL - LSL) / 6 sigma_within. Cpk = min(USL - mean, mean - LSL) / 3 sigma_within. Pp, Ppk use overall sigma. sigma_within = Rbar/d2 (Xbar-R), sbar/c4 (Xbar-S), MRbar/1.128 (I-MR).</t>
         </is>
       </c>
       <c r="C15" s="8" t="inlineStr">
         <is>
-          <t>Cpk &gt;= 1.33 capable; 1.00 to 1.33 marginal; &lt; 1.00 not capable. Requires a stable process first.</t>
+          <t>Cpk &gt;= 1.33 capable; 1.00 to 1.33 marginal; &lt; 1.00 not capable. Six Sigma goal Cp 2.0, Cpk 1.5. PPAP new process: Ppk &gt;= 1.67. Requires a stable process first.</t>
         </is>
       </c>
       <c r="D15" s="8" t="inlineStr">
@@ -1803,7 +1833,7 @@
       </c>
       <c r="B16" s="8" t="inlineStr">
         <is>
-          <t>DPMO = defects / (units x opportunities) x 10^6. Sigma level = NORM.S.INV(1 - DPMO/10^6) + 1.5.</t>
+          <t>DPMO = defects / (units x opportunities) x 10^6. Sigma level = 1.5 - NORM.S.INV(DPMO/10^6). Short-term sigma level = 3 Cpk.</t>
         </is>
       </c>
       <c r="C16" s="8" t="inlineStr">
@@ -1915,7 +1945,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="51" customHeight="1">
+    <row r="21" ht="66" customHeight="1">
       <c r="A21" s="28" t="inlineStr">
         <is>
           <t>FMEA</t>
@@ -1928,7 +1958,7 @@
       </c>
       <c r="C21" s="10" t="inlineStr">
         <is>
-          <t>Act on highest RPN or High Action Priority; any Severity 9 to 10 gets action regardless.</t>
+          <t>Act on highest RPN (AIAG 4th) or High AP, review Medium AP (AIAG-VDA 2019). House rule, stricter than AIAG-VDA: any Severity 9 to 10 gets an action or a documented justification.</t>
         </is>
       </c>
       <c r="D21" s="10" t="inlineStr">
@@ -1944,7 +1974,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="111" customHeight="1">
+    <row r="22" ht="171" customHeight="1">
       <c r="A22" s="28" t="inlineStr">
         <is>
           <t>Hypothesis testing</t>
@@ -1972,9 +2002,11 @@
           <t>One-sample t (CI and test) (IPS ch. 7)
 Two-sample t (Welch) (IPS ch. 7)
 Paired t (IPS ch. 7)
+Inference for proportions (IPS ch. 8)
 Chi-square test for two-way tables (IPS ch. 9)
 One-way ANOVA (IPS ch. 12)
-Nonparametric tests (IPS ch. 15)</t>
+Nonparametric tests (IPS ch. 15 (companion))
+Bootstrap and permutation tests (IPS ch. 16 (companion))</t>
         </is>
       </c>
     </row>
@@ -2071,7 +2103,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="51" customHeight="1">
+    <row r="27" ht="66" customHeight="1">
       <c r="A27" s="30" t="inlineStr">
         <is>
           <t>Design of experiments (2^k factorial)</t>
@@ -2079,7 +2111,7 @@
       </c>
       <c r="B27" s="12" t="inlineStr">
         <is>
-          <t>Effect = mean(Y at +) - mean(Y at -). Runs = 2^k (x replicates). ANOVA on effects.</t>
+          <t>Effect = mean(Y at +) - mean(Y at -); regression coefficient = effect / 2. Runs = 2^k (x replicates). ANOVA on effects.</t>
         </is>
       </c>
       <c r="C27" s="12" t="inlineStr">
@@ -2091,7 +2123,8 @@
         <is>
           <t>Modeling and simulation
 Optimization / search over a space
-Iteration</t>
+Iteration
+Testing and verification</t>
         </is>
       </c>
       <c r="E27" s="12" t="inlineStr">
@@ -2252,7 +2285,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="51" customHeight="1">
+    <row r="34" ht="66" customHeight="1">
       <c r="A34" s="32" t="inlineStr">
         <is>
           <t>Xbar-R and I-MR charts</t>
@@ -2260,12 +2293,12 @@
       </c>
       <c r="B34" s="14" t="inlineStr">
         <is>
-          <t>Xbar-R: UCL/LCL = Xbarbar +/- A2 Rbar; R: UCL = D4 Rbar, LCL = D3 Rbar. I-MR: x +/- 2.66 MRbar; MR UCL = 3.267 MRbar.</t>
+          <t>Xbar-R: UCL/LCL = Xbarbar +/- A2 Rbar; R: UCL = D4 Rbar, LCL = D3 Rbar. I-MR: xbar +/- 2.66 MRbar; MR: UCL = 3.267 MRbar, LCL = 0.</t>
         </is>
       </c>
       <c r="C34" s="14" t="inlineStr">
         <is>
-          <t>Western Electric: 1 point beyond 3 sigma; 2 of 3 beyond 2 sigma; 4 of 5 beyond 1 sigma; 8 in a row one side.</t>
+          <t>Western Electric: 1 point beyond 3 sigma; 2 of 3 consecutive beyond 2 sigma on the same side; 4 of 5 consecutive beyond 1 sigma on the same side; 8 consecutive on one side of the center line.</t>
         </is>
       </c>
       <c r="D34" s="14" t="inlineStr">
@@ -2898,7 +2931,7 @@
         <v>1</v>
       </c>
       <c r="E25" s="45" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F25" s="41" t="inlineStr"/>
       <c r="G25" s="41">
@@ -3276,7 +3309,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="36" customHeight="1">
+    <row r="12" ht="51" customHeight="1">
       <c r="A12" s="26" t="inlineStr">
         <is>
           <t>Gage R&amp;R (MSA, ANOVA method)</t>
@@ -3289,7 +3322,7 @@
       </c>
       <c r="C12" s="8" t="inlineStr">
         <is>
-          <t>%GRR = sigma_GRR / sigma_total x 100. ndc = 1.41 x sigma_part / sigma_GRR.</t>
+          <t>%GRR = sigma_GRR / sigma_total x 100. %GRR to tolerance = 6 sigma_GRR / (USL - LSL) x 100. ndc = 1.41 x sigma_part / sigma_GRR, truncated to an integer.</t>
         </is>
       </c>
       <c r="D12" s="8" t="inlineStr">
@@ -3308,7 +3341,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="36" customHeight="1">
+    <row r="13" ht="66" customHeight="1">
       <c r="A13" s="26" t="inlineStr">
         <is>
           <t>Attribute agreement analysis</t>
@@ -3326,7 +3359,7 @@
       </c>
       <c r="D13" s="8" t="inlineStr">
         <is>
-          <t>kappa &gt;= 0.75 good; 0.40 to 0.75 marginal; &lt; 0.40 poor.</t>
+          <t>kappa &gt;= 0.75 good; 0.40 to 0.75 marginal; &lt; 0.40 poor. AIAG: effectiveness &gt;= 90%, miss rate &lt;= 2%, false alarm &lt;= 5%. A chi-square test shows association, not agreement.</t>
         </is>
       </c>
       <c r="E13" s="8" t="inlineStr">
@@ -3340,7 +3373,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="36" customHeight="1">
+    <row r="14" ht="51" customHeight="1">
       <c r="A14" s="26" t="inlineStr">
         <is>
           <t>Normality check</t>
@@ -3358,7 +3391,7 @@
       </c>
       <c r="D14" s="8" t="inlineStr">
         <is>
-          <t>p &gt; alpha and a straight plot -&gt; treat as normal; else transform or go nonparametric.</t>
+          <t>p &gt; alpha means no evidence against normality; decide from the plot. Large n: rely on the plot. Small n: the test has little power.</t>
         </is>
       </c>
       <c r="E14" s="8" t="inlineStr">
@@ -3372,7 +3405,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="36" customHeight="1">
+    <row r="15" ht="66" customHeight="1">
       <c r="A15" s="26" t="inlineStr">
         <is>
           <t>Baseline capability</t>
@@ -3385,12 +3418,12 @@
       </c>
       <c r="C15" s="8" t="inlineStr">
         <is>
-          <t>Cp = (USL - LSL) / 6 sigma_within. Cpk = min(USL - mean, mean - LSL) / 3 sigma_within. Pp, Ppk use overall sigma.</t>
+          <t>Cp = (USL - LSL) / 6 sigma_within. Cpk = min(USL - mean, mean - LSL) / 3 sigma_within. Pp, Ppk use overall sigma. sigma_within = Rbar/d2 (Xbar-R), sbar/c4 (Xbar-S), MRbar/1.128 (I-MR).</t>
         </is>
       </c>
       <c r="D15" s="8" t="inlineStr">
         <is>
-          <t>Cpk &gt;= 1.33 capable; 1.00 to 1.33 marginal; &lt; 1.00 not capable. Requires a stable process first.</t>
+          <t>Cpk &gt;= 1.33 capable; 1.00 to 1.33 marginal; &lt; 1.00 not capable. Six Sigma goal Cp 2.0, Cpk 1.5. PPAP new process: Ppk &gt;= 1.67. Requires a stable process first.</t>
         </is>
       </c>
       <c r="E15" s="8" t="inlineStr">
@@ -3404,7 +3437,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="36" customHeight="1">
+    <row r="16" ht="51" customHeight="1">
       <c r="A16" s="26" t="inlineStr">
         <is>
           <t>DPMO and sigma level</t>
@@ -3417,7 +3450,7 @@
       </c>
       <c r="C16" s="8" t="inlineStr">
         <is>
-          <t>DPMO = defects / (units x opportunities) x 10^6. Sigma level = NORM.S.INV(1 - DPMO/10^6) + 1.5.</t>
+          <t>DPMO = defects / (units x opportunities) x 10^6. Sigma level = 1.5 - NORM.S.INV(DPMO/10^6). Short-term sigma level = 3 Cpk.</t>
         </is>
       </c>
       <c r="D16" s="8" t="inlineStr">
@@ -3539,7 +3572,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="36" customHeight="1">
+    <row r="21" ht="66" customHeight="1">
       <c r="A21" s="28" t="inlineStr">
         <is>
           <t>FMEA</t>
@@ -3557,7 +3590,7 @@
       </c>
       <c r="D21" s="10" t="inlineStr">
         <is>
-          <t>Act on highest RPN or High Action Priority; any Severity 9 to 10 gets action regardless.</t>
+          <t>Act on highest RPN (AIAG 4th) or High AP, review Medium AP (AIAG-VDA 2019). House rule, stricter than AIAG-VDA: any Severity 9 to 10 gets an action or a documented justification.</t>
         </is>
       </c>
       <c r="E21" s="10" t="inlineStr">
@@ -3719,7 +3752,7 @@
       </c>
       <c r="C27" s="12" t="inlineStr">
         <is>
-          <t>Effect = mean(Y at +) - mean(Y at -). Runs = 2^k (x replicates). ANOVA on effects.</t>
+          <t>Effect = mean(Y at +) - mean(Y at -); regression coefficient = effect / 2. Runs = 2^k (x replicates). ANOVA on effects.</t>
         </is>
       </c>
       <c r="D27" s="12" t="inlineStr">
@@ -3905,7 +3938,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="51" customHeight="1">
+    <row r="34" ht="66" customHeight="1">
       <c r="A34" s="32" t="inlineStr">
         <is>
           <t>Xbar-R and I-MR charts</t>
@@ -3918,12 +3951,12 @@
       </c>
       <c r="C34" s="14" t="inlineStr">
         <is>
-          <t>Xbar-R: UCL/LCL = Xbarbar +/- A2 Rbar; R: UCL = D4 Rbar, LCL = D3 Rbar. I-MR: x +/- 2.66 MRbar; MR UCL = 3.267 MRbar.</t>
+          <t>Xbar-R: UCL/LCL = Xbarbar +/- A2 Rbar; R: UCL = D4 Rbar, LCL = D3 Rbar. I-MR: xbar +/- 2.66 MRbar; MR: UCL = 3.267 MRbar, LCL = 0.</t>
         </is>
       </c>
       <c r="D34" s="14" t="inlineStr">
         <is>
-          <t>Western Electric: 1 point beyond 3 sigma; 2 of 3 beyond 2 sigma; 4 of 5 beyond 1 sigma; 8 in a row one side.</t>
+          <t>Western Electric: 1 point beyond 3 sigma; 2 of 3 consecutive beyond 2 sigma on the same side; 4 of 5 consecutive beyond 1 sigma on the same side; 8 consecutive on one side of the center line.</t>
         </is>
       </c>
       <c r="E34" s="14" t="inlineStr">
@@ -4104,7 +4137,7 @@
       </c>
       <c r="E2" s="34" t="inlineStr">
         <is>
-          <t>DMAIC phases</t>
+          <t>DMAIC phases (from tags)</t>
         </is>
       </c>
       <c r="F2" s="34" t="inlineStr">
@@ -4182,7 +4215,7 @@
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Measure, Analyze, Control</t>
+          <t>Define, Measure, Analyze, Control</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
@@ -4267,7 +4300,7 @@
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Measure, Improve, Control</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
@@ -4765,7 +4798,7 @@
       </c>
       <c r="E19" s="16" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Analyze</t>
         </is>
       </c>
       <c r="F19" s="16" t="inlineStr">
@@ -4955,7 +4988,7 @@
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>Analyze, Improve</t>
+          <t>Analyze</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr">
@@ -4969,7 +5002,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="51" customHeight="1">
+    <row r="25" ht="66" customHeight="1">
       <c r="A25" s="16" t="inlineStr">
         <is>
           <t>CT-TEST</t>
@@ -4992,13 +5025,14 @@
       </c>
       <c r="E25" s="16" t="inlineStr">
         <is>
-          <t>Measure, Improve</t>
+          <t>Measure, Analyze, Improve</t>
         </is>
       </c>
       <c r="F25" s="16" t="inlineStr">
         <is>
           <t>Gage R&amp;R (MSA, ANOVA method)
 Hypothesis testing
+Design of experiments (2^k factorial)
 Pilot and before/after test</t>
         </is>
       </c>
@@ -5145,7 +5179,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:G22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5266,7 +5300,7 @@
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>Use the normal table or NORM.S.DIST.</t>
+          <t>Use the normal table or NORM.S.DIST(z, TRUE).</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
@@ -5312,7 +5346,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="36" customHeight="1">
+    <row r="6" ht="66" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
           <t>ST-T1</t>
@@ -5330,7 +5364,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Random sample; normal or n &gt;= 30 without strong skew.</t>
+          <t>Random sample. IPS guideline: n &lt; 15 needs near-normal data; n &gt;= 15 unless outliers or strong skew; n &gt;= 40 is fine even if skewed.</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
@@ -5386,7 +5420,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="36" customHeight="1">
+    <row r="8" ht="66" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
           <t>ST-T2</t>
@@ -5404,7 +5438,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Independent random samples; each roughly normal or large.</t>
+          <t>Independent random samples. IPS guideline on n1 + n2: &lt; 15 near-normal; &gt;= 15 unless outliers or strong skew; &gt;= 40 even if skewed.</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
@@ -5423,7 +5457,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="36" customHeight="1">
+    <row r="9" ht="81" customHeight="1">
       <c r="A9" s="18" t="inlineStr">
         <is>
           <t>ST-PROP</t>
@@ -5441,12 +5475,12 @@
       </c>
       <c r="D9" s="18" t="inlineStr">
         <is>
-          <t>Counts of successes and failures &gt;= 10 (or use plus-four).</t>
+          <t>CI: successes and failures &gt;= 10 (each sample). Test: n p0 and n(1 - p0) &gt;= 10; two-sample test &gt;= 5 each. Plus-four: n &gt;= 10 (one sample) or &gt;= 5 each (two).</t>
         </is>
       </c>
       <c r="E9" s="18" t="inlineStr">
         <is>
-          <t>phat +/- z* sqrt(phat(1 - phat)/n). Two-proportion z with pooled p.</t>
+          <t>phat +/- z* sqrt(phat(1 - phat)/n). Two-proportion z: pooled p in the test SE, unpooled SE in the CI.</t>
         </is>
       </c>
       <c r="F9" s="18" t="inlineStr">
@@ -5460,7 +5494,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="36" customHeight="1">
+    <row r="10" ht="66" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
           <t>ST-CHI</t>
@@ -5478,7 +5512,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Expected counts mostly &gt;= 5.</t>
+          <t>2 x 2: all expected counts &gt;= 5. Larger tables: average expected &gt;= 5 and minimum &gt;= 1 (IPS). Otherwise Fisher's exact.</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
@@ -5648,190 +5682,227 @@
     <row r="15" ht="36" customHeight="1">
       <c r="A15" s="18" t="inlineStr">
         <is>
-          <t>ST-NP</t>
+          <t>ST-LOGIT</t>
         </is>
       </c>
       <c r="B15" s="49" t="inlineStr">
         <is>
-          <t>Nonparametric tests</t>
+          <t>Logistic regression</t>
         </is>
       </c>
       <c r="C15" s="18" t="inlineStr">
         <is>
-          <t>When normality fails and n is small.</t>
+          <t>Pass/fail Y vs continuous or several X.</t>
         </is>
       </c>
       <c r="D15" s="18" t="inlineStr">
         <is>
-          <t>Independent samples; similar shapes for location claims.</t>
+          <t>Independent trials; logit linear in X.</t>
         </is>
       </c>
       <c r="E15" s="18" t="inlineStr">
         <is>
-          <t>Wilcoxon rank sum, Wilcoxon signed rank, Kruskal-Wallis.</t>
+          <t>log(p / (1 - p)) = b0 + b1 x; odds ratio = e^b1.</t>
         </is>
       </c>
       <c r="F15" s="18" t="inlineStr">
         <is>
-          <t>Reject H0 when p &lt; alpha.</t>
+          <t>Slope significant when p &lt; alpha.</t>
         </is>
       </c>
       <c r="G15" s="18" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>14 (companion)</t>
         </is>
       </c>
     </row>
     <row r="16" ht="36" customHeight="1">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>ST-BOOT</t>
+          <t>ST-NP</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Bootstrap and permutation tests</t>
+          <t>Nonparametric tests</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>CIs and tests without distribution assumptions.</t>
+          <t>When normality fails and n is small.</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>Sample represents the population.</t>
+          <t>Independent samples; similar shapes for location claims.</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>Resample with replacement B &gt;= 1000 times; percentile CI.</t>
+          <t>Wilcoxon rank sum, Wilcoxon signed rank, Kruskal-Wallis.</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>Use when formulas do not apply.</t>
+          <t>Reject H0 when p &lt; alpha.</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>15 (companion)</t>
         </is>
       </c>
     </row>
     <row r="17" ht="36" customHeight="1">
       <c r="A17" s="18" t="inlineStr">
         <is>
-          <t>ST-POWER</t>
+          <t>ST-BOOT</t>
         </is>
       </c>
       <c r="B17" s="49" t="inlineStr">
         <is>
-          <t>Power and sample size</t>
+          <t>Bootstrap and permutation tests</t>
         </is>
       </c>
       <c r="C17" s="18" t="inlineStr">
         <is>
-          <t>Choose n before collecting data.</t>
+          <t>CIs and tests without distribution assumptions.</t>
         </is>
       </c>
       <c r="D17" s="18" t="inlineStr">
         <is>
-          <t>Planned effect size and sigma.</t>
+          <t>Sample represents the population.</t>
         </is>
       </c>
       <c r="E17" s="18" t="inlineStr">
         <is>
-          <t>Power = P(reject H0 | Ha true); pick n for power &gt;= 0.80.</t>
+          <t>Resample with replacement B &gt;= 1000 times; percentile CI.</t>
         </is>
       </c>
       <c r="F17" s="18" t="inlineStr">
         <is>
-          <t>Underpowered study: a non-significant result proves nothing.</t>
+          <t>Use when formulas do not apply.</t>
         </is>
       </c>
       <c r="G17" s="18" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>16 (companion)</t>
         </is>
       </c>
     </row>
     <row r="18" ht="36" customHeight="1">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>ST-SPC</t>
+          <t>ST-POWER</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Statistical process control</t>
+          <t>Power and sample size</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Monitor a process over time.</t>
+          <t>Choose n before collecting data.</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>Rational subgroups; Phase I establishes limits.</t>
+          <t>Planned effect size and sigma.</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>3-sigma control limits from within-subgroup variation.</t>
+          <t>Power = P(reject H0 | Ha true); pick n for power &gt;= 0.80.</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>Out-of-control signal triggers the reaction plan.</t>
+          <t>Underpowered study: a non-significant result proves nothing.</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>17 (companion)</t>
+          <t>6</t>
         </is>
       </c>
     </row>
     <row r="19" ht="36" customHeight="1">
       <c r="A19" s="18" t="inlineStr">
         <is>
+          <t>ST-SPC</t>
+        </is>
+      </c>
+      <c r="B19" s="49" t="inlineStr">
+        <is>
+          <t>Statistical process control</t>
+        </is>
+      </c>
+      <c r="C19" s="18" t="inlineStr">
+        <is>
+          <t>Monitor a process over time.</t>
+        </is>
+      </c>
+      <c r="D19" s="18" t="inlineStr">
+        <is>
+          <t>Rational subgroups; Phase I establishes limits.</t>
+        </is>
+      </c>
+      <c r="E19" s="18" t="inlineStr">
+        <is>
+          <t>3-sigma control limits from within-subgroup variation.</t>
+        </is>
+      </c>
+      <c r="F19" s="18" t="inlineStr">
+        <is>
+          <t>Out-of-control signal triggers the reaction plan.</t>
+        </is>
+      </c>
+      <c r="G19" s="18" t="inlineStr">
+        <is>
+          <t>17 (companion)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="36" customHeight="1">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
           <t>ST-CAP</t>
         </is>
       </c>
-      <c r="B19" s="49" t="inlineStr">
+      <c r="B20" s="3" t="inlineStr">
         <is>
           <t>Process capability</t>
         </is>
       </c>
-      <c r="C19" s="18" t="inlineStr">
+      <c r="C20" s="4" t="inlineStr">
         <is>
           <t>Compare process spread to spec.</t>
         </is>
       </c>
-      <c r="D19" s="18" t="inlineStr">
+      <c r="D20" s="4" t="inlineStr">
         <is>
           <t>Process in control; distribution known (often normal).</t>
         </is>
       </c>
-      <c r="E19" s="18" t="inlineStr">
+      <c r="E20" s="4" t="inlineStr">
         <is>
           <t>Cp, Cpk, Pp, Ppk (see Six Sigma sheet).</t>
         </is>
       </c>
-      <c r="F19" s="18" t="inlineStr">
+      <c r="F20" s="4" t="inlineStr">
         <is>
           <t>Compute only after control is shown.</t>
         </is>
       </c>
-      <c r="G19" s="18" t="inlineStr">
+      <c r="G20" s="4" t="inlineStr">
         <is>
           <t>17 (companion)</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="50" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="50" t="inlineStr">
         <is>
           <t>* Likely chapter in recent editions. Verify against the owner's edition; the stats-book extraction replaces this sheet.</t>
         </is>
@@ -5839,7 +5910,7 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A21:G21"/>
+    <mergeCell ref="A22:G22"/>
     <mergeCell ref="A1:G1"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
@@ -5862,7 +5933,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E35"/>
+  <dimension ref="A1:I54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -6021,7 +6092,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="21" customHeight="1">
+    <row r="8" ht="36" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
           <t>Continuous</t>
@@ -6044,11 +6115,11 @@
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>Transform or bootstrap (ST-BOOT)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="21" customHeight="1">
+          <t>Friedman (one block factor), aligned rank transform, or permutation / bootstrap (ST-BOOT)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="36" customHeight="1">
       <c r="A9" s="20" t="inlineStr">
         <is>
           <t>Continuous</t>
@@ -6056,22 +6127,22 @@
       </c>
       <c r="B9" s="20" t="inlineStr">
         <is>
-          <t>Continuous</t>
+          <t>Categorical</t>
         </is>
       </c>
       <c r="C9" s="20" t="inlineStr">
         <is>
-          <t>1 X</t>
+          <t>Compare spread, 2+ groups</t>
         </is>
       </c>
       <c r="D9" s="20" t="inlineStr">
         <is>
-          <t>Simple regression (ST-REG)</t>
+          <t>Levene or Bonett (software); F test only if normal (IPS warns it is not robust)</t>
         </is>
       </c>
       <c r="E9" s="20" t="inlineStr">
         <is>
-          <t>Spearman rank correlation</t>
+          <t>Permutation test on variances</t>
         </is>
       </c>
     </row>
@@ -6088,44 +6159,44 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>2+ X</t>
+          <t>1 X</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Multiple regression / DOE (ST-MREG)</t>
+          <t>Simple regression (ST-REG)</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>Bootstrap coefficients (ST-BOOT)</t>
+          <t>Spearman rank correlation</t>
         </is>
       </c>
     </row>
     <row r="11" ht="21" customHeight="1">
       <c r="A11" s="20" t="inlineStr">
         <is>
-          <t>Attribute (pass/fail)</t>
+          <t>Continuous</t>
         </is>
       </c>
       <c r="B11" s="20" t="inlineStr">
         <is>
-          <t>None (vs target)</t>
+          <t>Continuous</t>
         </is>
       </c>
       <c r="C11" s="20" t="inlineStr">
         <is>
-          <t>1 proportion</t>
+          <t>2+ X</t>
         </is>
       </c>
       <c r="D11" s="20" t="inlineStr">
         <is>
-          <t>One-proportion z (ST-PROP)</t>
+          <t>Multiple regression / DOE (ST-MREG)</t>
         </is>
       </c>
       <c r="E11" s="20" t="inlineStr">
         <is>
-          <t>Exact binomial test</t>
+          <t>Bootstrap coefficients (ST-BOOT)</t>
         </is>
       </c>
     </row>
@@ -6137,29 +6208,29 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Categorical</t>
+          <t>None (vs target)</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>2 groups</t>
+          <t>1 proportion</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Two-proportion z (ST-PROP)</t>
+          <t>One-proportion z (ST-PROP)</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>Fisher's exact test</t>
+          <t>Exact binomial test</t>
         </is>
       </c>
     </row>
     <row r="13" ht="21" customHeight="1">
       <c r="A13" s="20" t="inlineStr">
         <is>
-          <t>Attribute (counts)</t>
+          <t>Attribute (pass/fail)</t>
         </is>
       </c>
       <c r="B13" s="20" t="inlineStr">
@@ -6169,12 +6240,12 @@
       </c>
       <c r="C13" s="20" t="inlineStr">
         <is>
-          <t>2+ groups</t>
+          <t>2 groups</t>
         </is>
       </c>
       <c r="D13" s="20" t="inlineStr">
         <is>
-          <t>Chi-square two-way table (ST-CHI)</t>
+          <t>Two-proportion z (ST-PROP)</t>
         </is>
       </c>
       <c r="E13" s="20" t="inlineStr">
@@ -6191,504 +6262,1009 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
+          <t>Categorical</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>2 paired</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>McNemar</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>Exact binomial on discordant pairs</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="36" customHeight="1">
+      <c r="A15" s="20" t="inlineStr">
+        <is>
+          <t>Attribute (counts)</t>
+        </is>
+      </c>
+      <c r="B15" s="20" t="inlineStr">
+        <is>
+          <t>Categorical</t>
+        </is>
+      </c>
+      <c r="C15" s="20" t="inlineStr">
+        <is>
+          <t>2+ groups (pass/fail or multi-level)</t>
+        </is>
+      </c>
+      <c r="D15" s="20" t="inlineStr">
+        <is>
+          <t>Chi-square two-way table (ST-CHI)</t>
+        </is>
+      </c>
+      <c r="E15" s="20" t="inlineStr">
+        <is>
+          <t>Fisher's exact test</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="21" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Attribute (counts)</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>None (vs expected shares)</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>1 variable</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>Chi-square goodness of fit (ST-CHI)</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>Exact multinomial</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="21" customHeight="1">
+      <c r="A17" s="20" t="inlineStr">
+        <is>
+          <t>Defect counts per unit</t>
+        </is>
+      </c>
+      <c r="B17" s="20" t="inlineStr">
+        <is>
+          <t>Categorical</t>
+        </is>
+      </c>
+      <c r="C17" s="20" t="inlineStr">
+        <is>
+          <t>1 or 2 rates</t>
+        </is>
+      </c>
+      <c r="D17" s="20" t="inlineStr">
+        <is>
+          <t>Poisson rate test</t>
+        </is>
+      </c>
+      <c r="E17" s="20" t="inlineStr">
+        <is>
+          <t>Exact Poisson</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="21" customHeight="1">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Attribute (pass/fail)</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
           <t>Continuous</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
+      <c r="C18" s="4" t="inlineStr">
         <is>
           <t>1+ X</t>
         </is>
       </c>
-      <c r="D14" s="4" t="inlineStr">
-        <is>
-          <t>Logistic regression</t>
-        </is>
-      </c>
-      <c r="E14" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="24" customHeight="1">
-      <c r="A16" s="51" t="inlineStr">
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>Logistic regression (ST-LOGIT)</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>Exact logistic regression</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="24" customHeight="1">
+      <c r="A20" s="51" t="inlineStr">
         <is>
           <t>2. Control chart selection</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="32" customHeight="1">
-      <c r="A17" s="52" t="inlineStr">
+    <row r="21" ht="32" customHeight="1">
+      <c r="A21" s="52" t="inlineStr">
         <is>
           <t>Data type</t>
         </is>
       </c>
-      <c r="B17" s="52" t="inlineStr">
+      <c r="B21" s="52" t="inlineStr">
         <is>
           <t>Subgroup / sample</t>
         </is>
       </c>
-      <c r="C17" s="52" t="inlineStr">
+      <c r="C21" s="52" t="inlineStr">
         <is>
           <t>Chart</t>
         </is>
       </c>
-      <c r="D17" s="52" t="inlineStr">
+      <c r="D21" s="52" t="inlineStr">
         <is>
           <t>Control limits</t>
         </is>
       </c>
-      <c r="E17" s="52" t="inlineStr">
+      <c r="E21" s="52" t="inlineStr">
         <is>
           <t>Typical use</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="36" customHeight="1">
-      <c r="A18" s="4" t="inlineStr">
+    <row r="22" ht="36" customHeight="1">
+      <c r="A22" s="4" t="inlineStr">
         <is>
           <t>Continuous</t>
         </is>
       </c>
-      <c r="B18" s="4" t="inlineStr">
+      <c r="B22" s="4" t="inlineStr">
         <is>
           <t>n = 1</t>
         </is>
       </c>
-      <c r="C18" s="4" t="inlineStr">
+      <c r="C22" s="4" t="inlineStr">
         <is>
           <t>I-MR</t>
         </is>
       </c>
-      <c r="D18" s="4" t="inlineStr">
-        <is>
-          <t>x +/- 2.66 MRbar; MR UCL = 3.267 MRbar</t>
-        </is>
-      </c>
-      <c r="E18" s="4" t="inlineStr">
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>xbar +/- 2.66 MRbar; MR: UCL = 3.267 MRbar, LCL = 0</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
         <is>
           <t>One reading per period; slow or costly measurements.</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="21" customHeight="1">
-      <c r="A19" s="20" t="inlineStr">
+    <row r="23" ht="21" customHeight="1">
+      <c r="A23" s="20" t="inlineStr">
         <is>
           <t>Continuous</t>
         </is>
       </c>
-      <c r="B19" s="20" t="inlineStr">
+      <c r="B23" s="20" t="inlineStr">
         <is>
           <t>2 to 9</t>
         </is>
       </c>
-      <c r="C19" s="20" t="inlineStr">
+      <c r="C23" s="20" t="inlineStr">
         <is>
           <t>Xbar-R</t>
         </is>
       </c>
-      <c r="D19" s="20" t="inlineStr">
+      <c r="D23" s="20" t="inlineStr">
         <is>
           <t>Xbarbar +/- A2 Rbar; R: D3 Rbar to D4 Rbar</t>
         </is>
       </c>
-      <c r="E19" s="20" t="inlineStr">
+      <c r="E23" s="20" t="inlineStr">
         <is>
           <t>Small rational subgroups (most common).</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="36" customHeight="1">
-      <c r="A20" s="4" t="inlineStr">
+    <row r="24" ht="36" customHeight="1">
+      <c r="A24" s="4" t="inlineStr">
         <is>
           <t>Continuous</t>
         </is>
       </c>
-      <c r="B20" s="4" t="inlineStr">
+      <c r="B24" s="4" t="inlineStr">
         <is>
           <t>10 or more</t>
         </is>
       </c>
-      <c r="C20" s="4" t="inlineStr">
+      <c r="C24" s="4" t="inlineStr">
         <is>
           <t>Xbar-S</t>
         </is>
       </c>
-      <c r="D20" s="4" t="inlineStr">
+      <c r="D24" s="4" t="inlineStr">
         <is>
           <t>Xbarbar +/- A3 sbar; S: B3 sbar to B4 sbar</t>
         </is>
       </c>
-      <c r="E20" s="4" t="inlineStr">
+      <c r="E24" s="4" t="inlineStr">
         <is>
           <t>Large subgroups; s estimates spread better than R.</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="21" customHeight="1">
-      <c r="A21" s="20" t="inlineStr">
+    <row r="25" ht="36" customHeight="1">
+      <c r="A25" s="20" t="inlineStr">
         <is>
           <t>Defectives (pass/fail)</t>
         </is>
       </c>
-      <c r="B21" s="20" t="inlineStr">
+      <c r="B25" s="20" t="inlineStr">
         <is>
           <t>Constant n</t>
         </is>
       </c>
-      <c r="C21" s="20" t="inlineStr">
+      <c r="C25" s="20" t="inlineStr">
         <is>
           <t>np</t>
         </is>
       </c>
-      <c r="D21" s="20" t="inlineStr">
-        <is>
-          <t>n pbar +/- 3 sqrt(n pbar (1 - pbar))</t>
-        </is>
-      </c>
-      <c r="E21" s="20" t="inlineStr">
+      <c r="D25" s="20" t="inlineStr">
+        <is>
+          <t>n pbar +/- 3 sqrt(n pbar (1 - pbar)); LCL floors at 0</t>
+        </is>
+      </c>
+      <c r="E25" s="20" t="inlineStr">
         <is>
           <t>Count of defective units, fixed sample size.</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="21" customHeight="1">
-      <c r="A22" s="4" t="inlineStr">
+    <row r="26" ht="36" customHeight="1">
+      <c r="A26" s="4" t="inlineStr">
         <is>
           <t>Defectives (pass/fail)</t>
         </is>
       </c>
-      <c r="B22" s="4" t="inlineStr">
+      <c r="B26" s="4" t="inlineStr">
         <is>
           <t>Varying n</t>
         </is>
       </c>
-      <c r="C22" s="4" t="inlineStr">
+      <c r="C26" s="4" t="inlineStr">
         <is>
           <t>p</t>
         </is>
       </c>
-      <c r="D22" s="4" t="inlineStr">
-        <is>
-          <t>pbar +/- 3 sqrt(pbar (1 - pbar) / n_i)</t>
-        </is>
-      </c>
-      <c r="E22" s="4" t="inlineStr">
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>pbar +/- 3 sqrt(pbar (1 - pbar) / n_i); LCL floors at 0</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="inlineStr">
         <is>
           <t>Fraction defective; limits change with each n_i.</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="36" customHeight="1">
-      <c r="A23" s="20" t="inlineStr">
+    <row r="27" ht="36" customHeight="1">
+      <c r="A27" s="20" t="inlineStr">
         <is>
           <t>Defects (counts)</t>
         </is>
       </c>
-      <c r="B23" s="20" t="inlineStr">
+      <c r="B27" s="20" t="inlineStr">
         <is>
           <t>Constant area</t>
         </is>
       </c>
-      <c r="C23" s="20" t="inlineStr">
+      <c r="C27" s="20" t="inlineStr">
         <is>
           <t>c</t>
         </is>
       </c>
-      <c r="D23" s="20" t="inlineStr">
-        <is>
-          <t>cbar +/- 3 sqrt(cbar)</t>
-        </is>
-      </c>
-      <c r="E23" s="20" t="inlineStr">
+      <c r="D27" s="20" t="inlineStr">
+        <is>
+          <t>cbar +/- 3 sqrt(cbar); LCL floors at 0</t>
+        </is>
+      </c>
+      <c r="E27" s="20" t="inlineStr">
         <is>
           <t>Defects per unit, same inspection area each time.</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="21" customHeight="1">
-      <c r="A24" s="4" t="inlineStr">
+    <row r="28" ht="36" customHeight="1">
+      <c r="A28" s="4" t="inlineStr">
         <is>
           <t>Defects (counts)</t>
         </is>
       </c>
-      <c r="B24" s="4" t="inlineStr">
+      <c r="B28" s="4" t="inlineStr">
         <is>
           <t>Varying area</t>
         </is>
       </c>
-      <c r="C24" s="4" t="inlineStr">
+      <c r="C28" s="4" t="inlineStr">
         <is>
           <t>u</t>
         </is>
       </c>
-      <c r="D24" s="4" t="inlineStr">
-        <is>
-          <t>ubar +/- 3 sqrt(ubar / n_i)</t>
-        </is>
-      </c>
-      <c r="E24" s="4" t="inlineStr">
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>ubar +/- 3 sqrt(ubar / n_i); LCL floors at 0</t>
+        </is>
+      </c>
+      <c r="E28" s="4" t="inlineStr">
         <is>
           <t>Defects per unit when inspection area varies.</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="24" customHeight="1">
-      <c r="A26" s="51" t="inlineStr">
-        <is>
-          <t>3. Project loop with stop conditions and term limits</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="32" customHeight="1">
-      <c r="A27" s="52" t="inlineStr">
-        <is>
-          <t>Step</t>
-        </is>
-      </c>
-      <c r="B27" s="52" t="inlineStr">
-        <is>
-          <t>Action</t>
-        </is>
-      </c>
-      <c r="C27" s="52" t="inlineStr">
-        <is>
-          <t>Check</t>
-        </is>
-      </c>
-      <c r="D27" s="52" t="inlineStr">
-        <is>
-          <t>If yes, go to</t>
-        </is>
-      </c>
-      <c r="E27" s="52" t="inlineStr">
-        <is>
-          <t>If no, go to</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="51" customHeight="1">
-      <c r="A28" s="4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B28" s="4" t="inlineStr">
-        <is>
-          <t>Write the objective, metric, baseline, target, and done-when line.</t>
-        </is>
-      </c>
-      <c r="C28" s="4" t="inlineStr">
-        <is>
-          <t>All five written?</t>
-        </is>
-      </c>
-      <c r="D28" s="4" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="E28" s="4" t="inlineStr">
-        <is>
-          <t>Stop: ask the owner</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="51" customHeight="1">
+    <row r="29" ht="36" customHeight="1">
       <c r="A29" s="20" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>Defectives or defects</t>
         </is>
       </c>
       <c r="B29" s="20" t="inlineStr">
         <is>
-          <t>Set term limits: attempts (6), time budget, token budget.</t>
+          <t>Very large n, limits too tight</t>
         </is>
       </c>
       <c r="C29" s="20" t="inlineStr">
         <is>
-          <t>Limits written?</t>
+          <t>Laney p' / u'</t>
         </is>
       </c>
       <c r="D29" s="20" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>p or u limits x sigma_Z</t>
         </is>
       </c>
       <c r="E29" s="20" t="inlineStr">
         <is>
-          <t>Set defaults, then 3</t>
+          <t>Overdispersed attribute data.</t>
         </is>
       </c>
     </row>
     <row r="30" ht="36" customHeight="1">
       <c r="A30" s="4" t="inlineStr">
         <is>
+          <t>Continuous</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>Any; detect shifts &lt; 1.5 sigma</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>EWMA or CUSUM</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>Software (lambda, L or k, h)</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t>Small sustained shifts; complements a Shewhart chart.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="24" customHeight="1">
+      <c r="A32" s="51" t="inlineStr">
+        <is>
+          <t>2b. Control chart constants by subgroup size n</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="52" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="B33" s="52" t="inlineStr">
+        <is>
+          <t>A2</t>
+        </is>
+      </c>
+      <c r="C33" s="52" t="inlineStr">
+        <is>
+          <t>D3</t>
+        </is>
+      </c>
+      <c r="D33" s="52" t="inlineStr">
+        <is>
+          <t>D4</t>
+        </is>
+      </c>
+      <c r="E33" s="52" t="inlineStr">
+        <is>
+          <t>A3</t>
+        </is>
+      </c>
+      <c r="F33" s="52" t="inlineStr">
+        <is>
+          <t>B3</t>
+        </is>
+      </c>
+      <c r="G33" s="52" t="inlineStr">
+        <is>
+          <t>B4</t>
+        </is>
+      </c>
+      <c r="H33" s="52" t="inlineStr">
+        <is>
+          <t>d2</t>
+        </is>
+      </c>
+      <c r="I33" s="52" t="inlineStr">
+        <is>
+          <t>c4</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="53" t="n">
+        <v>2</v>
+      </c>
+      <c r="B34" s="54" t="n">
+        <v>1.88</v>
+      </c>
+      <c r="C34" s="54" t="n">
+        <v>0</v>
+      </c>
+      <c r="D34" s="54" t="n">
+        <v>3.267</v>
+      </c>
+      <c r="E34" s="54" t="n">
+        <v>2.659</v>
+      </c>
+      <c r="F34" s="54" t="n">
+        <v>0</v>
+      </c>
+      <c r="G34" s="54" t="n">
+        <v>3.267</v>
+      </c>
+      <c r="H34" s="54" t="n">
+        <v>1.128</v>
+      </c>
+      <c r="I34" s="55" t="n">
+        <v>0.7979000000000001</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="56" t="n">
+        <v>3</v>
+      </c>
+      <c r="B35" s="57" t="n">
+        <v>1.023</v>
+      </c>
+      <c r="C35" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="D35" s="57" t="n">
+        <v>2.574</v>
+      </c>
+      <c r="E35" s="57" t="n">
+        <v>1.954</v>
+      </c>
+      <c r="F35" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="G35" s="57" t="n">
+        <v>2.568</v>
+      </c>
+      <c r="H35" s="57" t="n">
+        <v>1.693</v>
+      </c>
+      <c r="I35" s="58" t="n">
+        <v>0.8862</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="53" t="n">
+        <v>4</v>
+      </c>
+      <c r="B36" s="54" t="n">
+        <v>0.729</v>
+      </c>
+      <c r="C36" s="54" t="n">
+        <v>0</v>
+      </c>
+      <c r="D36" s="54" t="n">
+        <v>2.282</v>
+      </c>
+      <c r="E36" s="54" t="n">
+        <v>1.628</v>
+      </c>
+      <c r="F36" s="54" t="n">
+        <v>0</v>
+      </c>
+      <c r="G36" s="54" t="n">
+        <v>2.266</v>
+      </c>
+      <c r="H36" s="54" t="n">
+        <v>2.059</v>
+      </c>
+      <c r="I36" s="55" t="n">
+        <v>0.9213</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="56" t="n">
+        <v>5</v>
+      </c>
+      <c r="B37" s="57" t="n">
+        <v>0.577</v>
+      </c>
+      <c r="C37" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="D37" s="57" t="n">
+        <v>2.114</v>
+      </c>
+      <c r="E37" s="57" t="n">
+        <v>1.427</v>
+      </c>
+      <c r="F37" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="G37" s="57" t="n">
+        <v>2.089</v>
+      </c>
+      <c r="H37" s="57" t="n">
+        <v>2.326</v>
+      </c>
+      <c r="I37" s="58" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="53" t="n">
+        <v>6</v>
+      </c>
+      <c r="B38" s="54" t="n">
+        <v>0.483</v>
+      </c>
+      <c r="C38" s="54" t="n">
+        <v>0</v>
+      </c>
+      <c r="D38" s="54" t="n">
+        <v>2.004</v>
+      </c>
+      <c r="E38" s="54" t="n">
+        <v>1.287</v>
+      </c>
+      <c r="F38" s="54" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="G38" s="54" t="n">
+        <v>1.97</v>
+      </c>
+      <c r="H38" s="54" t="n">
+        <v>2.534</v>
+      </c>
+      <c r="I38" s="55" t="n">
+        <v>0.9515</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="56" t="n">
+        <v>7</v>
+      </c>
+      <c r="B39" s="57" t="n">
+        <v>0.419</v>
+      </c>
+      <c r="C39" s="57" t="n">
+        <v>0.076</v>
+      </c>
+      <c r="D39" s="57" t="n">
+        <v>1.924</v>
+      </c>
+      <c r="E39" s="57" t="n">
+        <v>1.182</v>
+      </c>
+      <c r="F39" s="57" t="n">
+        <v>0.118</v>
+      </c>
+      <c r="G39" s="57" t="n">
+        <v>1.882</v>
+      </c>
+      <c r="H39" s="57" t="n">
+        <v>2.704</v>
+      </c>
+      <c r="I39" s="58" t="n">
+        <v>0.9594</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="53" t="n">
+        <v>8</v>
+      </c>
+      <c r="B40" s="54" t="n">
+        <v>0.373</v>
+      </c>
+      <c r="C40" s="54" t="n">
+        <v>0.136</v>
+      </c>
+      <c r="D40" s="54" t="n">
+        <v>1.864</v>
+      </c>
+      <c r="E40" s="54" t="n">
+        <v>1.099</v>
+      </c>
+      <c r="F40" s="54" t="n">
+        <v>0.185</v>
+      </c>
+      <c r="G40" s="54" t="n">
+        <v>1.815</v>
+      </c>
+      <c r="H40" s="54" t="n">
+        <v>2.847</v>
+      </c>
+      <c r="I40" s="55" t="n">
+        <v>0.965</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="56" t="n">
+        <v>9</v>
+      </c>
+      <c r="B41" s="57" t="n">
+        <v>0.337</v>
+      </c>
+      <c r="C41" s="57" t="n">
+        <v>0.184</v>
+      </c>
+      <c r="D41" s="57" t="n">
+        <v>1.816</v>
+      </c>
+      <c r="E41" s="57" t="n">
+        <v>1.032</v>
+      </c>
+      <c r="F41" s="57" t="n">
+        <v>0.239</v>
+      </c>
+      <c r="G41" s="57" t="n">
+        <v>1.761</v>
+      </c>
+      <c r="H41" s="57" t="n">
+        <v>2.97</v>
+      </c>
+      <c r="I41" s="58" t="n">
+        <v>0.9693000000000001</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="53" t="n">
+        <v>10</v>
+      </c>
+      <c r="B42" s="54" t="n">
+        <v>0.308</v>
+      </c>
+      <c r="C42" s="54" t="n">
+        <v>0.223</v>
+      </c>
+      <c r="D42" s="54" t="n">
+        <v>1.777</v>
+      </c>
+      <c r="E42" s="54" t="n">
+        <v>0.975</v>
+      </c>
+      <c r="F42" s="54" t="n">
+        <v>0.284</v>
+      </c>
+      <c r="G42" s="54" t="n">
+        <v>1.716</v>
+      </c>
+      <c r="H42" s="54" t="n">
+        <v>3.078</v>
+      </c>
+      <c r="I42" s="55" t="n">
+        <v>0.9727</v>
+      </c>
+    </row>
+    <row r="44" ht="24" customHeight="1">
+      <c r="A44" s="51" t="inlineStr">
+        <is>
+          <t>3. Project loop with stop conditions and term limits</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="32" customHeight="1">
+      <c r="A45" s="52" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="B45" s="52" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="C45" s="52" t="inlineStr">
+        <is>
+          <t>Check</t>
+        </is>
+      </c>
+      <c r="D45" s="52" t="inlineStr">
+        <is>
+          <t>If yes, go to</t>
+        </is>
+      </c>
+      <c r="E45" s="52" t="inlineStr">
+        <is>
+          <t>If no, go to</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="51" customHeight="1">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B46" s="4" t="inlineStr">
+        <is>
+          <t>Write the objective, metric, baseline, target, and done-when line.</t>
+        </is>
+      </c>
+      <c r="C46" s="4" t="inlineStr">
+        <is>
+          <t>All five written?</t>
+        </is>
+      </c>
+      <c r="D46" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E46" s="4" t="inlineStr">
+        <is>
+          <t>Stop: ask the owner</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="51" customHeight="1">
+      <c r="A47" s="20" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B47" s="20" t="inlineStr">
+        <is>
+          <t>Set term limits: attempts (6), time budget, token budget.</t>
+        </is>
+      </c>
+      <c r="C47" s="20" t="inlineStr">
+        <is>
+          <t>Limits written?</t>
+        </is>
+      </c>
+      <c r="D47" s="20" t="inlineStr">
+        <is>
           <t>3</t>
         </is>
       </c>
-      <c r="B30" s="4" t="inlineStr">
-        <is>
-          <t>Attempt the next sub-problem.</t>
-        </is>
-      </c>
-      <c r="C30" s="4" t="inlineStr">
-        <is>
-          <t>Done-when true?</t>
-        </is>
-      </c>
-      <c r="D30" s="4" t="inlineStr">
+      <c r="E47" s="20" t="inlineStr">
+        <is>
+          <t>Set defaults (6 attempts; time and token budgets as agreed with the owner), then 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="36" customHeight="1">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B48" s="4" t="inlineStr">
+        <is>
+          <t>Attempt the next sub-problem (attempts + 1).</t>
+        </is>
+      </c>
+      <c r="C48" s="4" t="inlineStr">
+        <is>
+          <t>Sub-problem done-when true?</t>
+        </is>
+      </c>
+      <c r="D48" s="4" t="inlineStr">
+        <is>
+          <t>3b</t>
+        </is>
+      </c>
+      <c r="E48" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="36" customHeight="1">
+      <c r="A49" s="20" t="inlineStr">
+        <is>
+          <t>3b</t>
+        </is>
+      </c>
+      <c r="B49" s="20" t="inlineStr">
+        <is>
+          <t>Check the whole project.</t>
+        </is>
+      </c>
+      <c r="C49" s="20" t="inlineStr">
+        <is>
+          <t>Project done-when true?</t>
+        </is>
+      </c>
+      <c r="D49" s="20" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="E30" s="4" t="inlineStr">
+      <c r="E49" s="20" t="inlineStr">
+        <is>
+          <t>5 (then next sub-problem)</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="51" customHeight="1">
+      <c r="A50" s="4" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-    </row>
-    <row r="31" ht="51" customHeight="1">
-      <c r="A31" s="20" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B31" s="20" t="inlineStr">
+      <c r="B50" s="4" t="inlineStr">
         <is>
           <t>Log the failure in FAILURES.xlsx (category, root cause).</t>
         </is>
       </c>
-      <c r="C31" s="20" t="inlineStr">
+      <c r="C50" s="4" t="inlineStr">
         <is>
           <t>Same root cause seen before?</t>
         </is>
       </c>
-      <c r="D31" s="20" t="inlineStr">
-        <is>
-          <t>Apply the logged fix, then 3</t>
-        </is>
-      </c>
-      <c r="E31" s="20" t="inlineStr">
+      <c r="D50" s="4" t="inlineStr">
+        <is>
+          <t>Apply the logged fix, then 5</t>
+        </is>
+      </c>
+      <c r="E50" s="4" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="21" customHeight="1">
-      <c r="A32" s="4" t="inlineStr">
+    <row r="51" ht="21" customHeight="1">
+      <c r="A51" s="20" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="B32" s="4" t="inlineStr">
+      <c r="B51" s="20" t="inlineStr">
         <is>
           <t>Check term limits.</t>
         </is>
       </c>
-      <c r="C32" s="4" t="inlineStr">
+      <c r="C51" s="20" t="inlineStr">
         <is>
           <t>Any limit reached?</t>
         </is>
       </c>
-      <c r="D32" s="4" t="inlineStr">
+      <c r="D51" s="20" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="E32" s="4" t="inlineStr">
+      <c r="E51" s="20" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="51" customHeight="1">
-      <c r="A33" s="20" t="inlineStr">
+    <row r="52" ht="51" customHeight="1">
+      <c r="A52" s="4" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="B33" s="20" t="inlineStr">
+      <c r="B52" s="4" t="inlineStr">
         <is>
           <t>Run Part B self-audit (objective, history, claim ledger, sweep).</t>
         </is>
       </c>
-      <c r="C33" s="20" t="inlineStr">
+      <c r="C52" s="4" t="inlineStr">
         <is>
           <t>Every claim verified?</t>
         </is>
       </c>
-      <c r="D33" s="20" t="inlineStr">
+      <c r="D52" s="4" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="E33" s="20" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="36" customHeight="1">
-      <c r="A34" s="4" t="inlineStr">
+      <c r="E52" s="4" t="inlineStr">
+        <is>
+          <t>4 (log as 'Claimed work not done')</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="36" customHeight="1">
+      <c r="A53" s="20" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="B34" s="4" t="inlineStr">
+      <c r="B53" s="20" t="inlineStr">
         <is>
           <t>Write the hand-off plan (B6).</t>
         </is>
       </c>
-      <c r="C34" s="4" t="inlineStr">
+      <c r="C53" s="20" t="inlineStr">
         <is>
           <t>A fresh agent could finish from it?</t>
         </is>
       </c>
-      <c r="D34" s="4" t="inlineStr">
+      <c r="D53" s="20" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="E34" s="4" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="36" customHeight="1">
-      <c r="A35" s="20" t="inlineStr">
+      <c r="E53" s="20" t="inlineStr">
+        <is>
+          <t>Revise once; if still no, list the missing items as the plan's first line, then 8</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="36" customHeight="1">
+      <c r="A54" s="4" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="B35" s="20" t="inlineStr">
+      <c r="B54" s="4" t="inlineStr">
         <is>
           <t>Run Parts C and D; report.</t>
         </is>
       </c>
-      <c r="C35" s="20" t="inlineStr">
+      <c r="C54" s="4" t="inlineStr">
         <is>
           <t>Report block complete?</t>
         </is>
       </c>
-      <c r="D35" s="20" t="inlineStr">
+      <c r="D54" s="4" t="inlineStr">
         <is>
           <t>End</t>
         </is>
       </c>
-      <c r="E35" s="20" t="inlineStr">
-        <is>
-          <t>8</t>
+      <c r="E54" s="4" t="inlineStr">
+        <is>
+          <t>Fill the missing block once; if still incomplete, mark it missing in the report, then End</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A16:E16"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A26:E26"/>
+  <mergeCells count="5">
+    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A32:I32"/>
+    <mergeCell ref="A44:I44"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A20:I20"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.4" right="0.4" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -6724,49 +7300,49 @@
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="53" t="inlineStr">
+      <c r="A1" s="59" t="inlineStr">
         <is>
           <t>Failure log: one row per failure, every project, every run</t>
         </is>
       </c>
     </row>
     <row r="2" ht="32" customHeight="1">
-      <c r="A2" s="54" t="inlineStr">
+      <c r="A2" s="60" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B2" s="54" t="inlineStr">
+      <c r="B2" s="60" t="inlineStr">
         <is>
           <t>Project</t>
         </is>
       </c>
-      <c r="C2" s="54" t="inlineStr">
+      <c r="C2" s="60" t="inlineStr">
         <is>
           <t>Agent</t>
         </is>
       </c>
-      <c r="D2" s="54" t="inlineStr">
+      <c r="D2" s="60" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="E2" s="54" t="inlineStr">
+      <c r="E2" s="60" t="inlineStr">
         <is>
           <t>What happened</t>
         </is>
       </c>
-      <c r="F2" s="54" t="inlineStr">
+      <c r="F2" s="60" t="inlineStr">
         <is>
           <t>Root cause</t>
         </is>
       </c>
-      <c r="G2" s="54" t="inlineStr">
+      <c r="G2" s="60" t="inlineStr">
         <is>
           <t>Fix / rule added</t>
         </is>
       </c>
-      <c r="H2" s="54" t="inlineStr">
+      <c r="H2" s="60" t="inlineStr">
         <is>
           <t>Recurrence (Y/N)</t>
         </is>
@@ -7025,204 +7601,204 @@
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="55" t="n"/>
-      <c r="B9" s="55" t="n"/>
-      <c r="C9" s="55" t="n"/>
-      <c r="D9" s="55" t="n"/>
-      <c r="E9" s="55" t="n"/>
-      <c r="F9" s="55" t="n"/>
-      <c r="G9" s="55" t="n"/>
-      <c r="H9" s="55" t="n"/>
+      <c r="A9" s="61" t="n"/>
+      <c r="B9" s="61" t="n"/>
+      <c r="C9" s="61" t="n"/>
+      <c r="D9" s="61" t="n"/>
+      <c r="E9" s="61" t="n"/>
+      <c r="F9" s="61" t="n"/>
+      <c r="G9" s="61" t="n"/>
+      <c r="H9" s="61" t="n"/>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="55" t="n"/>
-      <c r="B10" s="55" t="n"/>
-      <c r="C10" s="55" t="n"/>
-      <c r="D10" s="55" t="n"/>
-      <c r="E10" s="55" t="n"/>
-      <c r="F10" s="55" t="n"/>
-      <c r="G10" s="55" t="n"/>
-      <c r="H10" s="55" t="n"/>
+      <c r="A10" s="61" t="n"/>
+      <c r="B10" s="61" t="n"/>
+      <c r="C10" s="61" t="n"/>
+      <c r="D10" s="61" t="n"/>
+      <c r="E10" s="61" t="n"/>
+      <c r="F10" s="61" t="n"/>
+      <c r="G10" s="61" t="n"/>
+      <c r="H10" s="61" t="n"/>
     </row>
     <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="55" t="n"/>
-      <c r="B11" s="55" t="n"/>
-      <c r="C11" s="55" t="n"/>
-      <c r="D11" s="55" t="n"/>
-      <c r="E11" s="55" t="n"/>
-      <c r="F11" s="55" t="n"/>
-      <c r="G11" s="55" t="n"/>
-      <c r="H11" s="55" t="n"/>
+      <c r="A11" s="61" t="n"/>
+      <c r="B11" s="61" t="n"/>
+      <c r="C11" s="61" t="n"/>
+      <c r="D11" s="61" t="n"/>
+      <c r="E11" s="61" t="n"/>
+      <c r="F11" s="61" t="n"/>
+      <c r="G11" s="61" t="n"/>
+      <c r="H11" s="61" t="n"/>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="55" t="n"/>
-      <c r="B12" s="55" t="n"/>
-      <c r="C12" s="55" t="n"/>
-      <c r="D12" s="55" t="n"/>
-      <c r="E12" s="55" t="n"/>
-      <c r="F12" s="55" t="n"/>
-      <c r="G12" s="55" t="n"/>
-      <c r="H12" s="55" t="n"/>
+      <c r="A12" s="61" t="n"/>
+      <c r="B12" s="61" t="n"/>
+      <c r="C12" s="61" t="n"/>
+      <c r="D12" s="61" t="n"/>
+      <c r="E12" s="61" t="n"/>
+      <c r="F12" s="61" t="n"/>
+      <c r="G12" s="61" t="n"/>
+      <c r="H12" s="61" t="n"/>
     </row>
     <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="55" t="n"/>
-      <c r="B13" s="55" t="n"/>
-      <c r="C13" s="55" t="n"/>
-      <c r="D13" s="55" t="n"/>
-      <c r="E13" s="55" t="n"/>
-      <c r="F13" s="55" t="n"/>
-      <c r="G13" s="55" t="n"/>
-      <c r="H13" s="55" t="n"/>
+      <c r="A13" s="61" t="n"/>
+      <c r="B13" s="61" t="n"/>
+      <c r="C13" s="61" t="n"/>
+      <c r="D13" s="61" t="n"/>
+      <c r="E13" s="61" t="n"/>
+      <c r="F13" s="61" t="n"/>
+      <c r="G13" s="61" t="n"/>
+      <c r="H13" s="61" t="n"/>
     </row>
     <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="55" t="n"/>
-      <c r="B14" s="55" t="n"/>
-      <c r="C14" s="55" t="n"/>
-      <c r="D14" s="55" t="n"/>
-      <c r="E14" s="55" t="n"/>
-      <c r="F14" s="55" t="n"/>
-      <c r="G14" s="55" t="n"/>
-      <c r="H14" s="55" t="n"/>
+      <c r="A14" s="61" t="n"/>
+      <c r="B14" s="61" t="n"/>
+      <c r="C14" s="61" t="n"/>
+      <c r="D14" s="61" t="n"/>
+      <c r="E14" s="61" t="n"/>
+      <c r="F14" s="61" t="n"/>
+      <c r="G14" s="61" t="n"/>
+      <c r="H14" s="61" t="n"/>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="55" t="n"/>
-      <c r="B15" s="55" t="n"/>
-      <c r="C15" s="55" t="n"/>
-      <c r="D15" s="55" t="n"/>
-      <c r="E15" s="55" t="n"/>
-      <c r="F15" s="55" t="n"/>
-      <c r="G15" s="55" t="n"/>
-      <c r="H15" s="55" t="n"/>
+      <c r="A15" s="61" t="n"/>
+      <c r="B15" s="61" t="n"/>
+      <c r="C15" s="61" t="n"/>
+      <c r="D15" s="61" t="n"/>
+      <c r="E15" s="61" t="n"/>
+      <c r="F15" s="61" t="n"/>
+      <c r="G15" s="61" t="n"/>
+      <c r="H15" s="61" t="n"/>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="55" t="n"/>
-      <c r="B16" s="55" t="n"/>
-      <c r="C16" s="55" t="n"/>
-      <c r="D16" s="55" t="n"/>
-      <c r="E16" s="55" t="n"/>
-      <c r="F16" s="55" t="n"/>
-      <c r="G16" s="55" t="n"/>
-      <c r="H16" s="55" t="n"/>
+      <c r="A16" s="61" t="n"/>
+      <c r="B16" s="61" t="n"/>
+      <c r="C16" s="61" t="n"/>
+      <c r="D16" s="61" t="n"/>
+      <c r="E16" s="61" t="n"/>
+      <c r="F16" s="61" t="n"/>
+      <c r="G16" s="61" t="n"/>
+      <c r="H16" s="61" t="n"/>
     </row>
     <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="55" t="n"/>
-      <c r="B17" s="55" t="n"/>
-      <c r="C17" s="55" t="n"/>
-      <c r="D17" s="55" t="n"/>
-      <c r="E17" s="55" t="n"/>
-      <c r="F17" s="55" t="n"/>
-      <c r="G17" s="55" t="n"/>
-      <c r="H17" s="55" t="n"/>
+      <c r="A17" s="61" t="n"/>
+      <c r="B17" s="61" t="n"/>
+      <c r="C17" s="61" t="n"/>
+      <c r="D17" s="61" t="n"/>
+      <c r="E17" s="61" t="n"/>
+      <c r="F17" s="61" t="n"/>
+      <c r="G17" s="61" t="n"/>
+      <c r="H17" s="61" t="n"/>
     </row>
     <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="55" t="n"/>
-      <c r="B18" s="55" t="n"/>
-      <c r="C18" s="55" t="n"/>
-      <c r="D18" s="55" t="n"/>
-      <c r="E18" s="55" t="n"/>
-      <c r="F18" s="55" t="n"/>
-      <c r="G18" s="55" t="n"/>
-      <c r="H18" s="55" t="n"/>
+      <c r="A18" s="61" t="n"/>
+      <c r="B18" s="61" t="n"/>
+      <c r="C18" s="61" t="n"/>
+      <c r="D18" s="61" t="n"/>
+      <c r="E18" s="61" t="n"/>
+      <c r="F18" s="61" t="n"/>
+      <c r="G18" s="61" t="n"/>
+      <c r="H18" s="61" t="n"/>
     </row>
     <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="55" t="n"/>
-      <c r="B19" s="55" t="n"/>
-      <c r="C19" s="55" t="n"/>
-      <c r="D19" s="55" t="n"/>
-      <c r="E19" s="55" t="n"/>
-      <c r="F19" s="55" t="n"/>
-      <c r="G19" s="55" t="n"/>
-      <c r="H19" s="55" t="n"/>
+      <c r="A19" s="61" t="n"/>
+      <c r="B19" s="61" t="n"/>
+      <c r="C19" s="61" t="n"/>
+      <c r="D19" s="61" t="n"/>
+      <c r="E19" s="61" t="n"/>
+      <c r="F19" s="61" t="n"/>
+      <c r="G19" s="61" t="n"/>
+      <c r="H19" s="61" t="n"/>
     </row>
     <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="55" t="n"/>
-      <c r="B20" s="55" t="n"/>
-      <c r="C20" s="55" t="n"/>
-      <c r="D20" s="55" t="n"/>
-      <c r="E20" s="55" t="n"/>
-      <c r="F20" s="55" t="n"/>
-      <c r="G20" s="55" t="n"/>
-      <c r="H20" s="55" t="n"/>
+      <c r="A20" s="61" t="n"/>
+      <c r="B20" s="61" t="n"/>
+      <c r="C20" s="61" t="n"/>
+      <c r="D20" s="61" t="n"/>
+      <c r="E20" s="61" t="n"/>
+      <c r="F20" s="61" t="n"/>
+      <c r="G20" s="61" t="n"/>
+      <c r="H20" s="61" t="n"/>
     </row>
     <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="55" t="n"/>
-      <c r="B21" s="55" t="n"/>
-      <c r="C21" s="55" t="n"/>
-      <c r="D21" s="55" t="n"/>
-      <c r="E21" s="55" t="n"/>
-      <c r="F21" s="55" t="n"/>
-      <c r="G21" s="55" t="n"/>
-      <c r="H21" s="55" t="n"/>
+      <c r="A21" s="61" t="n"/>
+      <c r="B21" s="61" t="n"/>
+      <c r="C21" s="61" t="n"/>
+      <c r="D21" s="61" t="n"/>
+      <c r="E21" s="61" t="n"/>
+      <c r="F21" s="61" t="n"/>
+      <c r="G21" s="61" t="n"/>
+      <c r="H21" s="61" t="n"/>
     </row>
     <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="55" t="n"/>
-      <c r="B22" s="55" t="n"/>
-      <c r="C22" s="55" t="n"/>
-      <c r="D22" s="55" t="n"/>
-      <c r="E22" s="55" t="n"/>
-      <c r="F22" s="55" t="n"/>
-      <c r="G22" s="55" t="n"/>
-      <c r="H22" s="55" t="n"/>
+      <c r="A22" s="61" t="n"/>
+      <c r="B22" s="61" t="n"/>
+      <c r="C22" s="61" t="n"/>
+      <c r="D22" s="61" t="n"/>
+      <c r="E22" s="61" t="n"/>
+      <c r="F22" s="61" t="n"/>
+      <c r="G22" s="61" t="n"/>
+      <c r="H22" s="61" t="n"/>
     </row>
     <row r="23" ht="20" customHeight="1">
-      <c r="A23" s="55" t="n"/>
-      <c r="B23" s="55" t="n"/>
-      <c r="C23" s="55" t="n"/>
-      <c r="D23" s="55" t="n"/>
-      <c r="E23" s="55" t="n"/>
-      <c r="F23" s="55" t="n"/>
-      <c r="G23" s="55" t="n"/>
-      <c r="H23" s="55" t="n"/>
+      <c r="A23" s="61" t="n"/>
+      <c r="B23" s="61" t="n"/>
+      <c r="C23" s="61" t="n"/>
+      <c r="D23" s="61" t="n"/>
+      <c r="E23" s="61" t="n"/>
+      <c r="F23" s="61" t="n"/>
+      <c r="G23" s="61" t="n"/>
+      <c r="H23" s="61" t="n"/>
     </row>
     <row r="24" ht="20" customHeight="1">
-      <c r="A24" s="55" t="n"/>
-      <c r="B24" s="55" t="n"/>
-      <c r="C24" s="55" t="n"/>
-      <c r="D24" s="55" t="n"/>
-      <c r="E24" s="55" t="n"/>
-      <c r="F24" s="55" t="n"/>
-      <c r="G24" s="55" t="n"/>
-      <c r="H24" s="55" t="n"/>
+      <c r="A24" s="61" t="n"/>
+      <c r="B24" s="61" t="n"/>
+      <c r="C24" s="61" t="n"/>
+      <c r="D24" s="61" t="n"/>
+      <c r="E24" s="61" t="n"/>
+      <c r="F24" s="61" t="n"/>
+      <c r="G24" s="61" t="n"/>
+      <c r="H24" s="61" t="n"/>
     </row>
     <row r="25" ht="20" customHeight="1">
-      <c r="A25" s="55" t="n"/>
-      <c r="B25" s="55" t="n"/>
-      <c r="C25" s="55" t="n"/>
-      <c r="D25" s="55" t="n"/>
-      <c r="E25" s="55" t="n"/>
-      <c r="F25" s="55" t="n"/>
-      <c r="G25" s="55" t="n"/>
-      <c r="H25" s="55" t="n"/>
+      <c r="A25" s="61" t="n"/>
+      <c r="B25" s="61" t="n"/>
+      <c r="C25" s="61" t="n"/>
+      <c r="D25" s="61" t="n"/>
+      <c r="E25" s="61" t="n"/>
+      <c r="F25" s="61" t="n"/>
+      <c r="G25" s="61" t="n"/>
+      <c r="H25" s="61" t="n"/>
     </row>
     <row r="26" ht="20" customHeight="1">
-      <c r="A26" s="55" t="n"/>
-      <c r="B26" s="55" t="n"/>
-      <c r="C26" s="55" t="n"/>
-      <c r="D26" s="55" t="n"/>
-      <c r="E26" s="55" t="n"/>
-      <c r="F26" s="55" t="n"/>
-      <c r="G26" s="55" t="n"/>
-      <c r="H26" s="55" t="n"/>
+      <c r="A26" s="61" t="n"/>
+      <c r="B26" s="61" t="n"/>
+      <c r="C26" s="61" t="n"/>
+      <c r="D26" s="61" t="n"/>
+      <c r="E26" s="61" t="n"/>
+      <c r="F26" s="61" t="n"/>
+      <c r="G26" s="61" t="n"/>
+      <c r="H26" s="61" t="n"/>
     </row>
     <row r="27" ht="20" customHeight="1">
-      <c r="A27" s="55" t="n"/>
-      <c r="B27" s="55" t="n"/>
-      <c r="C27" s="55" t="n"/>
-      <c r="D27" s="55" t="n"/>
-      <c r="E27" s="55" t="n"/>
-      <c r="F27" s="55" t="n"/>
-      <c r="G27" s="55" t="n"/>
-      <c r="H27" s="55" t="n"/>
+      <c r="A27" s="61" t="n"/>
+      <c r="B27" s="61" t="n"/>
+      <c r="C27" s="61" t="n"/>
+      <c r="D27" s="61" t="n"/>
+      <c r="E27" s="61" t="n"/>
+      <c r="F27" s="61" t="n"/>
+      <c r="G27" s="61" t="n"/>
+      <c r="H27" s="61" t="n"/>
     </row>
     <row r="28" ht="20" customHeight="1">
-      <c r="A28" s="55" t="n"/>
-      <c r="B28" s="55" t="n"/>
-      <c r="C28" s="55" t="n"/>
-      <c r="D28" s="55" t="n"/>
-      <c r="E28" s="55" t="n"/>
-      <c r="F28" s="55" t="n"/>
-      <c r="G28" s="55" t="n"/>
-      <c r="H28" s="55" t="n"/>
+      <c r="A28" s="61" t="n"/>
+      <c r="B28" s="61" t="n"/>
+      <c r="C28" s="61" t="n"/>
+      <c r="D28" s="61" t="n"/>
+      <c r="E28" s="61" t="n"/>
+      <c r="F28" s="61" t="n"/>
+      <c r="G28" s="61" t="n"/>
+      <c r="H28" s="61" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -7253,7 +7829,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col hidden="1" width="8" customWidth="1" min="1" max="1"/>
@@ -7266,425 +7842,436 @@
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="53" t="inlineStr">
+      <c r="A1" s="59" t="inlineStr">
         <is>
           <t>Failure Pareto: work the categories that reach 80% first</t>
         </is>
       </c>
     </row>
     <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="56" t="inlineStr">
+      <c r="A2" s="62" t="inlineStr">
         <is>
           <t>Counts update from the Failure Log. Columns A and D are hidden helpers. Add a category in toolbox_data.py.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="32" customHeight="1">
-      <c r="A3" s="54" t="inlineStr">
+      <c r="A3" s="60" t="inlineStr">
         <is>
           <t>Rank key</t>
         </is>
       </c>
-      <c r="B3" s="54" t="inlineStr">
+      <c r="B3" s="60" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="C3" s="54" t="inlineStr">
+      <c r="C3" s="60" t="inlineStr">
         <is>
           <t>Count</t>
         </is>
       </c>
-      <c r="D3" s="54" t="inlineStr">
+      <c r="D3" s="60" t="inlineStr">
         <is>
           <t>Rank</t>
         </is>
       </c>
-      <c r="E3" s="54" t="inlineStr">
+      <c r="E3" s="60" t="inlineStr">
         <is>
           <t>Category (sorted by count)</t>
         </is>
       </c>
-      <c r="F3" s="54" t="inlineStr">
+      <c r="F3" s="60" t="inlineStr">
         <is>
           <t>Count</t>
         </is>
       </c>
-      <c r="G3" s="54" t="inlineStr">
+      <c r="G3" s="60" t="inlineStr">
         <is>
           <t>Cumulative %</t>
         </is>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="57">
+      <c r="A4" s="63">
         <f>C4-ROW()/1000</f>
         <v/>
       </c>
-      <c r="B4" s="57" t="inlineStr">
+      <c r="B4" s="63" t="inlineStr">
         <is>
           <t>Claimed work not done</t>
         </is>
       </c>
-      <c r="C4" s="58">
+      <c r="C4" s="64">
         <f>COUNTIF('Failure Log'!$D$3:$D$502,B4)</f>
         <v/>
       </c>
-      <c r="D4" s="58">
+      <c r="D4" s="64">
         <f>RANK(A4,$A$4:$A$15)</f>
         <v/>
       </c>
-      <c r="E4" s="57">
+      <c r="E4" s="63">
         <f>INDEX($B$4:$B$15,MATCH(1,$D$4:$D$15,0))</f>
         <v/>
       </c>
-      <c r="F4" s="58">
+      <c r="F4" s="64">
         <f>INDEX($C$4:$C$15,MATCH(1,$D$4:$D$15,0))</f>
         <v/>
       </c>
-      <c r="G4" s="59">
+      <c r="G4" s="65">
         <f>IF(SUM($C$4:$C$15)=0,0,SUM($F$4:F4)/SUM($C$4:$C$15))</f>
         <v/>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="60">
+      <c r="A5" s="66">
         <f>C5-ROW()/1000</f>
         <v/>
       </c>
-      <c r="B5" s="60" t="inlineStr">
+      <c r="B5" s="66" t="inlineStr">
         <is>
           <t>Absence treated as proof</t>
         </is>
       </c>
-      <c r="C5" s="61">
+      <c r="C5" s="67">
         <f>COUNTIF('Failure Log'!$D$3:$D$502,B5)</f>
         <v/>
       </c>
-      <c r="D5" s="61">
+      <c r="D5" s="67">
         <f>RANK(A5,$A$4:$A$15)</f>
         <v/>
       </c>
-      <c r="E5" s="60">
+      <c r="E5" s="66">
         <f>INDEX($B$4:$B$15,MATCH(2,$D$4:$D$15,0))</f>
         <v/>
       </c>
-      <c r="F5" s="61">
+      <c r="F5" s="67">
         <f>INDEX($C$4:$C$15,MATCH(2,$D$4:$D$15,0))</f>
         <v/>
       </c>
-      <c r="G5" s="62">
+      <c r="G5" s="68">
         <f>IF(SUM($C$4:$C$15)=0,0,SUM($F$4:F5)/SUM($C$4:$C$15))</f>
         <v/>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="57">
+      <c r="A6" s="63">
         <f>C6-ROW()/1000</f>
         <v/>
       </c>
-      <c r="B6" s="57" t="inlineStr">
+      <c r="B6" s="63" t="inlineStr">
         <is>
           <t>Unknown left in a table</t>
         </is>
       </c>
-      <c r="C6" s="58">
+      <c r="C6" s="64">
         <f>COUNTIF('Failure Log'!$D$3:$D$502,B6)</f>
         <v/>
       </c>
-      <c r="D6" s="58">
+      <c r="D6" s="64">
         <f>RANK(A6,$A$4:$A$15)</f>
         <v/>
       </c>
-      <c r="E6" s="57">
+      <c r="E6" s="63">
         <f>INDEX($B$4:$B$15,MATCH(3,$D$4:$D$15,0))</f>
         <v/>
       </c>
-      <c r="F6" s="58">
+      <c r="F6" s="64">
         <f>INDEX($C$4:$C$15,MATCH(3,$D$4:$D$15,0))</f>
         <v/>
       </c>
-      <c r="G6" s="59">
+      <c r="G6" s="65">
         <f>IF(SUM($C$4:$C$15)=0,0,SUM($F$4:F6)/SUM($C$4:$C$15))</f>
         <v/>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="60">
+      <c r="A7" s="66">
         <f>C7-ROW()/1000</f>
         <v/>
       </c>
-      <c r="B7" s="60" t="inlineStr">
+      <c r="B7" s="66" t="inlineStr">
         <is>
           <t>Objective drift</t>
         </is>
       </c>
-      <c r="C7" s="61">
+      <c r="C7" s="67">
         <f>COUNTIF('Failure Log'!$D$3:$D$502,B7)</f>
         <v/>
       </c>
-      <c r="D7" s="61">
+      <c r="D7" s="67">
         <f>RANK(A7,$A$4:$A$15)</f>
         <v/>
       </c>
-      <c r="E7" s="60">
+      <c r="E7" s="66">
         <f>INDEX($B$4:$B$15,MATCH(4,$D$4:$D$15,0))</f>
         <v/>
       </c>
-      <c r="F7" s="61">
+      <c r="F7" s="67">
         <f>INDEX($C$4:$C$15,MATCH(4,$D$4:$D$15,0))</f>
         <v/>
       </c>
-      <c r="G7" s="62">
+      <c r="G7" s="68">
         <f>IF(SUM($C$4:$C$15)=0,0,SUM($F$4:F7)/SUM($C$4:$C$15))</f>
         <v/>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="57">
+      <c r="A8" s="63">
         <f>C8-ROW()/1000</f>
         <v/>
       </c>
-      <c r="B8" s="57" t="inlineStr">
+      <c r="B8" s="63" t="inlineStr">
         <is>
           <t>Exit attempt / premature stop</t>
         </is>
       </c>
-      <c r="C8" s="58">
+      <c r="C8" s="64">
         <f>COUNTIF('Failure Log'!$D$3:$D$502,B8)</f>
         <v/>
       </c>
-      <c r="D8" s="58">
+      <c r="D8" s="64">
         <f>RANK(A8,$A$4:$A$15)</f>
         <v/>
       </c>
-      <c r="E8" s="57">
+      <c r="E8" s="63">
         <f>INDEX($B$4:$B$15,MATCH(5,$D$4:$D$15,0))</f>
         <v/>
       </c>
-      <c r="F8" s="58">
+      <c r="F8" s="64">
         <f>INDEX($C$4:$C$15,MATCH(5,$D$4:$D$15,0))</f>
         <v/>
       </c>
-      <c r="G8" s="59">
+      <c r="G8" s="65">
         <f>IF(SUM($C$4:$C$15)=0,0,SUM($F$4:F8)/SUM($C$4:$C$15))</f>
         <v/>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="60">
+      <c r="A9" s="66">
         <f>C9-ROW()/1000</f>
         <v/>
       </c>
-      <c r="B9" s="60" t="inlineStr">
+      <c r="B9" s="66" t="inlineStr">
         <is>
           <t>Unreadable image or CAD view</t>
         </is>
       </c>
-      <c r="C9" s="61">
+      <c r="C9" s="67">
         <f>COUNTIF('Failure Log'!$D$3:$D$502,B9)</f>
         <v/>
       </c>
-      <c r="D9" s="61">
+      <c r="D9" s="67">
         <f>RANK(A9,$A$4:$A$15)</f>
         <v/>
       </c>
-      <c r="E9" s="60">
+      <c r="E9" s="66">
         <f>INDEX($B$4:$B$15,MATCH(6,$D$4:$D$15,0))</f>
         <v/>
       </c>
-      <c r="F9" s="61">
+      <c r="F9" s="67">
         <f>INDEX($C$4:$C$15,MATCH(6,$D$4:$D$15,0))</f>
         <v/>
       </c>
-      <c r="G9" s="62">
+      <c r="G9" s="68">
         <f>IF(SUM($C$4:$C$15)=0,0,SUM($F$4:F9)/SUM($C$4:$C$15))</f>
         <v/>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="57">
+      <c r="A10" s="63">
         <f>C10-ROW()/1000</f>
         <v/>
       </c>
-      <c r="B10" s="57" t="inlineStr">
+      <c r="B10" s="63" t="inlineStr">
         <is>
           <t>Math or unit error</t>
         </is>
       </c>
-      <c r="C10" s="58">
+      <c r="C10" s="64">
         <f>COUNTIF('Failure Log'!$D$3:$D$502,B10)</f>
         <v/>
       </c>
-      <c r="D10" s="58">
+      <c r="D10" s="64">
         <f>RANK(A10,$A$4:$A$15)</f>
         <v/>
       </c>
-      <c r="E10" s="57">
+      <c r="E10" s="63">
         <f>INDEX($B$4:$B$15,MATCH(7,$D$4:$D$15,0))</f>
         <v/>
       </c>
-      <c r="F10" s="58">
+      <c r="F10" s="64">
         <f>INDEX($C$4:$C$15,MATCH(7,$D$4:$D$15,0))</f>
         <v/>
       </c>
-      <c r="G10" s="59">
+      <c r="G10" s="65">
         <f>IF(SUM($C$4:$C$15)=0,0,SUM($F$4:F10)/SUM($C$4:$C$15))</f>
         <v/>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="60">
+      <c r="A11" s="66">
         <f>C11-ROW()/1000</f>
         <v/>
       </c>
-      <c r="B11" s="60" t="inlineStr">
+      <c r="B11" s="66" t="inlineStr">
         <is>
           <t>Unsourced value</t>
         </is>
       </c>
-      <c r="C11" s="61">
+      <c r="C11" s="67">
         <f>COUNTIF('Failure Log'!$D$3:$D$502,B11)</f>
         <v/>
       </c>
-      <c r="D11" s="61">
+      <c r="D11" s="67">
         <f>RANK(A11,$A$4:$A$15)</f>
         <v/>
       </c>
-      <c r="E11" s="60">
+      <c r="E11" s="66">
         <f>INDEX($B$4:$B$15,MATCH(8,$D$4:$D$15,0))</f>
         <v/>
       </c>
-      <c r="F11" s="61">
+      <c r="F11" s="67">
         <f>INDEX($C$4:$C$15,MATCH(8,$D$4:$D$15,0))</f>
         <v/>
       </c>
-      <c r="G11" s="62">
+      <c r="G11" s="68">
         <f>IF(SUM($C$4:$C$15)=0,0,SUM($F$4:F11)/SUM($C$4:$C$15))</f>
         <v/>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="57">
+      <c r="A12" s="63">
         <f>C12-ROW()/1000</f>
         <v/>
       </c>
-      <c r="B12" s="57" t="inlineStr">
+      <c r="B12" s="63" t="inlineStr">
         <is>
           <t>Artifact not secured / not pushed</t>
         </is>
       </c>
-      <c r="C12" s="58">
+      <c r="C12" s="64">
         <f>COUNTIF('Failure Log'!$D$3:$D$502,B12)</f>
         <v/>
       </c>
-      <c r="D12" s="58">
+      <c r="D12" s="64">
         <f>RANK(A12,$A$4:$A$15)</f>
         <v/>
       </c>
-      <c r="E12" s="57">
+      <c r="E12" s="63">
         <f>INDEX($B$4:$B$15,MATCH(9,$D$4:$D$15,0))</f>
         <v/>
       </c>
-      <c r="F12" s="58">
+      <c r="F12" s="64">
         <f>INDEX($C$4:$C$15,MATCH(9,$D$4:$D$15,0))</f>
         <v/>
       </c>
-      <c r="G12" s="59">
+      <c r="G12" s="65">
         <f>IF(SUM($C$4:$C$15)=0,0,SUM($F$4:F12)/SUM($C$4:$C$15))</f>
         <v/>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="60">
+      <c r="A13" s="66">
         <f>C13-ROW()/1000</f>
         <v/>
       </c>
-      <c r="B13" s="60" t="inlineStr">
+      <c r="B13" s="66" t="inlineStr">
         <is>
           <t>Wrong location / duplicate created</t>
         </is>
       </c>
-      <c r="C13" s="61">
+      <c r="C13" s="67">
         <f>COUNTIF('Failure Log'!$D$3:$D$502,B13)</f>
         <v/>
       </c>
-      <c r="D13" s="61">
+      <c r="D13" s="67">
         <f>RANK(A13,$A$4:$A$15)</f>
         <v/>
       </c>
-      <c r="E13" s="60">
+      <c r="E13" s="66">
         <f>INDEX($B$4:$B$15,MATCH(10,$D$4:$D$15,0))</f>
         <v/>
       </c>
-      <c r="F13" s="61">
+      <c r="F13" s="67">
         <f>INDEX($C$4:$C$15,MATCH(10,$D$4:$D$15,0))</f>
         <v/>
       </c>
-      <c r="G13" s="62">
+      <c r="G13" s="68">
         <f>IF(SUM($C$4:$C$15)=0,0,SUM($F$4:F13)/SUM($C$4:$C$15))</f>
         <v/>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="57">
+      <c r="A14" s="63">
         <f>C14-ROW()/1000</f>
         <v/>
       </c>
-      <c r="B14" s="57" t="inlineStr">
+      <c r="B14" s="63" t="inlineStr">
         <is>
           <t>Skill or procedure skipped</t>
         </is>
       </c>
-      <c r="C14" s="58">
+      <c r="C14" s="64">
         <f>COUNTIF('Failure Log'!$D$3:$D$502,B14)</f>
         <v/>
       </c>
-      <c r="D14" s="58">
+      <c r="D14" s="64">
         <f>RANK(A14,$A$4:$A$15)</f>
         <v/>
       </c>
-      <c r="E14" s="57">
+      <c r="E14" s="63">
         <f>INDEX($B$4:$B$15,MATCH(11,$D$4:$D$15,0))</f>
         <v/>
       </c>
-      <c r="F14" s="58">
+      <c r="F14" s="64">
         <f>INDEX($C$4:$C$15,MATCH(11,$D$4:$D$15,0))</f>
         <v/>
       </c>
-      <c r="G14" s="59">
+      <c r="G14" s="65">
         <f>IF(SUM($C$4:$C$15)=0,0,SUM($F$4:F14)/SUM($C$4:$C$15))</f>
         <v/>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="60">
+      <c r="A15" s="66">
         <f>C15-ROW()/1000</f>
         <v/>
       </c>
-      <c r="B15" s="60" t="inlineStr">
+      <c r="B15" s="66" t="inlineStr">
         <is>
           <t>Tool or environment failure</t>
         </is>
       </c>
-      <c r="C15" s="61">
+      <c r="C15" s="67">
         <f>COUNTIF('Failure Log'!$D$3:$D$502,B15)</f>
         <v/>
       </c>
-      <c r="D15" s="61">
+      <c r="D15" s="67">
         <f>RANK(A15,$A$4:$A$15)</f>
         <v/>
       </c>
-      <c r="E15" s="60">
+      <c r="E15" s="66">
         <f>INDEX($B$4:$B$15,MATCH(12,$D$4:$D$15,0))</f>
         <v/>
       </c>
-      <c r="F15" s="61">
+      <c r="F15" s="67">
         <f>INDEX($C$4:$C$15,MATCH(12,$D$4:$D$15,0))</f>
         <v/>
       </c>
-      <c r="G15" s="62">
+      <c r="G15" s="68">
         <f>IF(SUM($C$4:$C$15)=0,0,SUM($F$4:F15)/SUM($C$4:$C$15))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="69" t="inlineStr">
+        <is>
+          <t>Uncategorized log rows (must read 0)</t>
+        </is>
+      </c>
+      <c r="C16" s="70">
+        <f>COUNTA('Failure Log'!$D$3:$D$502)-SUM($C$4:$C$15)</f>
         <v/>
       </c>
     </row>

</xml_diff>